<commit_message>
Add spend metrics to ad aggregation and reports
Co-authored-by: mail135797 <mail135797@gmail.com>
</commit_message>
<xml_diff>
--- a/first_data.xlsx
+++ b/first_data.xlsx
@@ -481,16 +481,16 @@
         <v>5</v>
       </c>
       <c r="B2" s="2">
+        <v>19405664</v>
+      </c>
+      <c r="C2" s="2">
         <v>14151762</v>
       </c>
-      <c r="C2" s="2">
-        <v>19405664</v>
-      </c>
       <c r="D2" s="2">
-        <v>5253902</v>
+        <v>-5253902</v>
       </c>
       <c r="E2" s="3">
-        <v>1.371254265016611</v>
+        <v>0.7292593543823082</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -498,16 +498,16 @@
         <v>6</v>
       </c>
       <c r="B3" s="2">
+        <v>1270756.11</v>
+      </c>
+      <c r="C3" s="2">
         <v>1126374.84</v>
       </c>
-      <c r="C3" s="2">
-        <v>1270756.11</v>
-      </c>
       <c r="D3" s="2">
-        <v>144381.2700000003</v>
+        <v>-144381.2700000003</v>
       </c>
       <c r="E3" s="3">
-        <v>1.128182257693185</v>
+        <v>0.8863816047282274</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -515,16 +515,16 @@
         <v>7</v>
       </c>
       <c r="B4" s="4">
+        <v>0.06548377370648076</v>
+      </c>
+      <c r="C4" s="4">
         <v>0.07959255109010453</v>
       </c>
-      <c r="C4" s="4">
-        <v>0.06548377370648076</v>
-      </c>
       <c r="D4" s="4">
-        <v>-0.01410877738362377</v>
+        <v>0.01410877738362377</v>
       </c>
       <c r="E4" s="3">
-        <v>0.8227374648709072</v>
+        <v>1.215454555915849</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -532,16 +532,16 @@
         <v>8</v>
       </c>
       <c r="B5" s="2">
+        <v>4284016</v>
+      </c>
+      <c r="C5" s="2">
         <v>2804694</v>
       </c>
-      <c r="C5" s="2">
-        <v>4284016</v>
-      </c>
       <c r="D5" s="2">
-        <v>1479322</v>
+        <v>-1479322</v>
       </c>
       <c r="E5" s="3">
-        <v>1.527445061742921</v>
+        <v>0.6546880310437683</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -549,16 +549,16 @@
         <v>9</v>
       </c>
       <c r="B6" s="4">
+        <v>0.2207611138686107</v>
+      </c>
+      <c r="C6" s="4">
         <v>0.1981869112835561</v>
       </c>
-      <c r="C6" s="4">
-        <v>0.2207611138686107</v>
-      </c>
       <c r="D6" s="4">
-        <v>0.02257420258505466</v>
+        <v>-0.02257420258505466</v>
       </c>
       <c r="E6" s="3">
-        <v>1.113903599581087</v>
+        <v>0.8977437548240944</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -566,16 +566,16 @@
         <v>10</v>
       </c>
       <c r="B7" s="2">
+        <v>3013259.89</v>
+      </c>
+      <c r="C7" s="2">
         <v>1678319.16</v>
       </c>
-      <c r="C7" s="2">
-        <v>3013259.89</v>
-      </c>
       <c r="D7" s="2">
-        <v>1334940.73</v>
+        <v>-1334940.73</v>
       </c>
       <c r="E7" s="3">
-        <v>1.795403378461102</v>
+        <v>0.5569778981128641</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -583,16 +583,16 @@
         <v>11</v>
       </c>
       <c r="B8" s="3">
+        <v>3.371233839670462</v>
+      </c>
+      <c r="C8" s="3">
         <v>2.490018331730492</v>
       </c>
-      <c r="C8" s="3">
-        <v>3.371233839670462</v>
-      </c>
       <c r="D8" s="3">
-        <v>0.8812155079399693</v>
+        <v>-0.8812155079399693</v>
       </c>
       <c r="E8" s="3">
-        <v>1.353899204961897</v>
+        <v>0.7386074209476646</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -600,16 +600,16 @@
         <v>12</v>
       </c>
       <c r="B9" s="2">
+        <v>1614807</v>
+      </c>
+      <c r="C9" s="2">
         <v>1152079</v>
       </c>
-      <c r="C9" s="2">
-        <v>1614807</v>
-      </c>
       <c r="D9" s="2">
-        <v>462728</v>
+        <v>-462728</v>
       </c>
       <c r="E9" s="3">
-        <v>1.401646067674179</v>
+        <v>0.713446870121321</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -617,16 +617,16 @@
         <v>13</v>
       </c>
       <c r="B10" s="2">
+        <v>9418</v>
+      </c>
+      <c r="C10" s="2">
         <v>7070</v>
       </c>
-      <c r="C10" s="2">
-        <v>9418</v>
-      </c>
       <c r="D10" s="2">
-        <v>2348</v>
+        <v>-2348</v>
       </c>
       <c r="E10" s="3">
-        <v>1.332107496463932</v>
+        <v>0.7506901677638564</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -634,16 +634,16 @@
         <v>14</v>
       </c>
       <c r="B11" s="4">
+        <v>0.005832275931427099</v>
+      </c>
+      <c r="C11" s="4">
         <v>0.006136731942861557</v>
       </c>
-      <c r="C11" s="4">
-        <v>0.005832275931427099</v>
-      </c>
       <c r="D11" s="4">
-        <v>-0.0003044560114344582</v>
+        <v>0.0003044560114344582</v>
       </c>
       <c r="E11" s="3">
-        <v>0.950387924017341</v>
+        <v>1.052201921687879</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -651,16 +651,16 @@
         <v>15</v>
       </c>
       <c r="B12" s="2">
+        <v>158.0965971459934</v>
+      </c>
+      <c r="C12" s="2">
         <v>107.735438419927</v>
       </c>
-      <c r="C12" s="2">
-        <v>158.0965971459934</v>
-      </c>
       <c r="D12" s="2">
-        <v>50.36115872606636</v>
+        <v>-50.36115872606636</v>
       </c>
       <c r="E12" s="3">
-        <v>1.467452116635666</v>
+        <v>0.6814532403909956</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -668,16 +668,16 @@
         <v>16</v>
       </c>
       <c r="B13" s="2">
+        <v>134.928446591633</v>
+      </c>
+      <c r="C13" s="2">
         <v>159.3175162659123</v>
       </c>
-      <c r="C13" s="2">
-        <v>134.928446591633</v>
-      </c>
       <c r="D13" s="2">
-        <v>-24.38906967427923</v>
+        <v>24.38906967427923</v>
       </c>
       <c r="E13" s="3">
-        <v>0.8469153282959035</v>
+        <v>1.180755580386202</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -685,16 +685,16 @@
         <v>17</v>
       </c>
       <c r="B14" s="2">
+        <v>3801</v>
+      </c>
+      <c r="C14" s="2">
         <v>2982</v>
       </c>
-      <c r="C14" s="2">
-        <v>3801</v>
-      </c>
       <c r="D14" s="2">
-        <v>819</v>
+        <v>-819</v>
       </c>
       <c r="E14" s="3">
-        <v>1.274647887323944</v>
+        <v>0.7845303867403315</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -702,16 +702,16 @@
         <v>18</v>
       </c>
       <c r="B15" s="4">
+        <v>0.08919091102144829</v>
+      </c>
+      <c r="C15" s="4">
         <v>0.06944837340876944</v>
       </c>
-      <c r="C15" s="4">
-        <v>0.08919091102144829</v>
-      </c>
       <c r="D15" s="4">
-        <v>0.01974253761267884</v>
+        <v>-0.01974253761267884</v>
       </c>
       <c r="E15" s="3">
-        <v>1.284276458088879</v>
+        <v>0.7786485485283222</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -719,16 +719,16 @@
         <v>19</v>
       </c>
       <c r="B16" s="2">
+        <v>5105.41015522231</v>
+      </c>
+      <c r="C16" s="2">
         <v>4745.728370221328</v>
       </c>
-      <c r="C16" s="2">
-        <v>5105.41015522231</v>
-      </c>
       <c r="D16" s="2">
-        <v>359.681785000982</v>
+        <v>-359.681785000982</v>
       </c>
       <c r="E16" s="3">
-        <v>1.075790638852811</v>
+        <v>0.9295488953746323</v>
       </c>
     </row>
     <row r="17" spans="1:5">

</xml_diff>

<commit_message>
Refactor ads aggregation and input file detection
Update ads aggregation logic to use SP search term reports. Improve input file detection for traffic and ads reports.

Co-authored-by: mail135797 <mail135797@gmail.com>
</commit_message>
<xml_diff>
--- a/first_data.xlsx
+++ b/first_data.xlsx
@@ -481,16 +481,16 @@
         <v>5</v>
       </c>
       <c r="B2" s="2">
+        <v>14151762</v>
+      </c>
+      <c r="C2" s="2">
         <v>19405664</v>
       </c>
-      <c r="C2" s="2">
-        <v>14151762</v>
-      </c>
       <c r="D2" s="2">
-        <v>-5253902</v>
+        <v>5253902</v>
       </c>
       <c r="E2" s="3">
-        <v>0.7292593543823082</v>
+        <v>1.371254265016611</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -498,16 +498,16 @@
         <v>6</v>
       </c>
       <c r="B3" s="2">
-        <v>1270756.11</v>
+        <v>1370884.87</v>
       </c>
       <c r="C3" s="2">
-        <v>1126374.84</v>
+        <v>1099928.28</v>
       </c>
       <c r="D3" s="2">
-        <v>-144381.2700000003</v>
+        <v>-270956.5900000001</v>
       </c>
       <c r="E3" s="3">
-        <v>0.8863816047282274</v>
+        <v>0.8023491279760057</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -515,16 +515,16 @@
         <v>7</v>
       </c>
       <c r="B4" s="4">
-        <v>0.06548377370648076</v>
+        <v>0.09687026039584327</v>
       </c>
       <c r="C4" s="4">
-        <v>0.07959255109010453</v>
+        <v>0.0566807855685845</v>
       </c>
       <c r="D4" s="4">
-        <v>0.01410877738362377</v>
+        <v>-0.04018947482725877</v>
       </c>
       <c r="E4" s="3">
-        <v>1.215454555915849</v>
+        <v>0.5851206070569899</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -532,16 +532,16 @@
         <v>8</v>
       </c>
       <c r="B5" s="2">
-        <v>4284016</v>
+        <v>4339684</v>
       </c>
       <c r="C5" s="2">
-        <v>2804694</v>
+        <v>2653004</v>
       </c>
       <c r="D5" s="2">
-        <v>-1479322</v>
+        <v>-1686680</v>
       </c>
       <c r="E5" s="3">
-        <v>0.6546880310437683</v>
+        <v>0.611335756244003</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -549,16 +549,16 @@
         <v>9</v>
       </c>
       <c r="B6" s="4">
-        <v>0.2207611138686107</v>
+        <v>0.3066532633886861</v>
       </c>
       <c r="C6" s="4">
-        <v>0.1981869112835561</v>
+        <v>0.1367128689850551</v>
       </c>
       <c r="D6" s="4">
-        <v>-0.02257420258505466</v>
+        <v>-0.1699403944036311</v>
       </c>
       <c r="E6" s="3">
-        <v>0.8977437548240944</v>
+        <v>0.4458223189093218</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -566,16 +566,16 @@
         <v>10</v>
       </c>
       <c r="B7" s="2">
-        <v>3013259.89</v>
+        <v>2968799.13</v>
       </c>
       <c r="C7" s="2">
-        <v>1678319.16</v>
+        <v>1553075.72</v>
       </c>
       <c r="D7" s="2">
-        <v>-1334940.73</v>
+        <v>-1415723.41</v>
       </c>
       <c r="E7" s="3">
-        <v>0.5569778981128641</v>
+        <v>0.5231326378083384</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -583,16 +583,16 @@
         <v>11</v>
       </c>
       <c r="B8" s="3">
-        <v>3.371233839670462</v>
+        <v>3.165607918628499</v>
       </c>
       <c r="C8" s="3">
-        <v>2.490018331730492</v>
+        <v>2.411979079217784</v>
       </c>
       <c r="D8" s="3">
-        <v>-0.8812155079399693</v>
+        <v>-0.7536288394107156</v>
       </c>
       <c r="E8" s="3">
-        <v>0.7386074209476646</v>
+        <v>0.7619323495572927</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -600,16 +600,16 @@
         <v>12</v>
       </c>
       <c r="B9" s="2">
-        <v>1614807</v>
+        <v>502354</v>
       </c>
       <c r="C9" s="2">
-        <v>1152079</v>
+        <v>275205</v>
       </c>
       <c r="D9" s="2">
-        <v>-462728</v>
+        <v>-227149</v>
       </c>
       <c r="E9" s="3">
-        <v>0.713446870121321</v>
+        <v>0.5478308125345872</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -617,16 +617,16 @@
         <v>13</v>
       </c>
       <c r="B10" s="2">
-        <v>9418</v>
+        <v>10019</v>
       </c>
       <c r="C10" s="2">
-        <v>7070</v>
+        <v>6850</v>
       </c>
       <c r="D10" s="2">
-        <v>-2348</v>
+        <v>-3169</v>
       </c>
       <c r="E10" s="3">
-        <v>0.7506901677638564</v>
+        <v>0.6837009681604951</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -634,16 +634,16 @@
         <v>14</v>
       </c>
       <c r="B11" s="4">
-        <v>0.005832275931427099</v>
+        <v>0.01994410316231184</v>
       </c>
       <c r="C11" s="4">
-        <v>0.006136731942861557</v>
+        <v>0.02489053614578223</v>
       </c>
       <c r="D11" s="4">
-        <v>0.0003044560114344582</v>
+        <v>0.004946432983470399</v>
       </c>
       <c r="E11" s="3">
-        <v>1.052201921687879</v>
+        <v>1.248014811356252</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -651,16 +651,16 @@
         <v>15</v>
       </c>
       <c r="B12" s="2">
-        <v>158.0965971459934</v>
+        <v>0</v>
       </c>
       <c r="C12" s="2">
-        <v>107.735438419927</v>
+        <v>0</v>
       </c>
       <c r="D12" s="2">
-        <v>-50.36115872606636</v>
+        <v>0</v>
       </c>
       <c r="E12" s="3">
-        <v>0.6814532403909956</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -668,16 +668,16 @@
         <v>16</v>
       </c>
       <c r="B13" s="2">
-        <v>134.928446591633</v>
+        <v>136.8285128256313</v>
       </c>
       <c r="C13" s="2">
-        <v>159.3175162659123</v>
+        <v>160.5734715328467</v>
       </c>
       <c r="D13" s="2">
-        <v>24.38906967427923</v>
+        <v>23.7449587072154</v>
       </c>
       <c r="E13" s="3">
-        <v>1.180755580386202</v>
+        <v>1.173538089517022</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -685,16 +685,16 @@
         <v>17</v>
       </c>
       <c r="B14" s="2">
+        <v>2982</v>
+      </c>
+      <c r="C14" s="2">
         <v>3801</v>
       </c>
-      <c r="C14" s="2">
-        <v>2982</v>
-      </c>
       <c r="D14" s="2">
-        <v>-819</v>
+        <v>819</v>
       </c>
       <c r="E14" s="3">
-        <v>0.7845303867403315</v>
+        <v>1.274647887323944</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -702,16 +702,16 @@
         <v>18</v>
       </c>
       <c r="B15" s="4">
-        <v>0.08919091102144829</v>
+        <v>0.08743387563629104</v>
       </c>
       <c r="C15" s="4">
-        <v>0.06944837340876944</v>
+        <v>0.06613138686131387</v>
       </c>
       <c r="D15" s="4">
-        <v>-0.01974253761267884</v>
+        <v>-0.02130248877497717</v>
       </c>
       <c r="E15" s="3">
-        <v>0.7786485485283222</v>
+        <v>0.7563588641135887</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -719,16 +719,16 @@
         <v>19</v>
       </c>
       <c r="B16" s="2">
+        <v>4745.728370221328</v>
+      </c>
+      <c r="C16" s="2">
         <v>5105.41015522231</v>
       </c>
-      <c r="C16" s="2">
-        <v>4745.728370221328</v>
-      </c>
       <c r="D16" s="2">
-        <v>-359.681785000982</v>
+        <v>359.681785000982</v>
       </c>
       <c r="E16" s="3">
-        <v>0.9295488953746323</v>
+        <v>1.075790638852811</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -736,16 +736,16 @@
         <v>20</v>
       </c>
       <c r="B17" s="2">
-        <v>79</v>
+        <v>16</v>
       </c>
       <c r="C17" s="2">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D17" s="2">
-        <v>0</v>
+        <v>-14</v>
       </c>
       <c r="E17" s="3">
-        <v>1</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -753,16 +753,16 @@
         <v>21</v>
       </c>
       <c r="B18" s="2">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C18" s="2">
-        <v>76</v>
+        <v>11</v>
       </c>
       <c r="D18" s="2">
-        <v>0</v>
+        <v>-60</v>
       </c>
       <c r="E18" s="3">
-        <v>1</v>
+        <v>0.1549295774647887</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -770,16 +770,16 @@
         <v>22</v>
       </c>
       <c r="B19" s="2">
-        <v>557</v>
+        <v>62</v>
       </c>
       <c r="C19" s="2">
-        <v>557</v>
+        <v>34</v>
       </c>
       <c r="D19" s="2">
-        <v>0</v>
+        <v>-28</v>
       </c>
       <c r="E19" s="3">
-        <v>1</v>
+        <v>0.5483870967741935</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -787,16 +787,16 @@
         <v>23</v>
       </c>
       <c r="B20" s="2">
-        <v>33998</v>
+        <v>450</v>
       </c>
       <c r="C20" s="2">
-        <v>33998</v>
+        <v>383</v>
       </c>
       <c r="D20" s="2">
-        <v>0</v>
+        <v>-67</v>
       </c>
       <c r="E20" s="3">
-        <v>1</v>
+        <v>0.8511111111111112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>